<commit_message>
[20260310_115400_vd_ingame_masterdata_generation] ブロック基礎設計 vd_chi_boss_00001 / vd_osh_normal_00001 / vd_chi_normal_00001 追加
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/domain/tasks/20260310_115400_vd_ingame_masterdata_generation/vd-ingame-creator/vd_chi_normal_00001/vd_chi_normal_00001.xlsx
+++ b/domain/tasks/20260310_115400_vd_ingame_masterdata_generation/vd-ingame-creator/vd_chi_normal_00001/vd_chi_normal_00001.xlsx
@@ -1022,7 +1022,7 @@
       </c>
       <c r="F15" s="27" t="inlineStr">
         <is>
-          <t>0.50 / 0.50</t>
+          <t>0.5 / 0.5</t>
         </is>
       </c>
       <c r="G15" s="2" t="n"/>
@@ -1280,7 +1280,7 @@
       </c>
       <c r="I26" s="27" t="inlineStr">
         <is>
-          <t>雑魚（チェンソーマン固有敵）</t>
+          <t>雑魚</t>
         </is>
       </c>
       <c r="J26" s="2" t="n"/>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="I27" s="27" t="inlineStr">
         <is>
-          <t>雑魚（共通敵）</t>
+          <t>雑魚（共通）</t>
         </is>
       </c>
       <c r="J27" s="2" t="n"/>
@@ -1569,7 +1569,7 @@
       </c>
       <c r="H40" s="27" t="inlineStr">
         <is>
-          <t>開幕5体・序盤の圧力</t>
+          <t>開幕5体・序盤の壁役</t>
         </is>
       </c>
       <c r="I40" s="2" t="n"/>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H41" s="27" t="inlineStr">
         <is>
-          <t>1.5秒後・属性変化で変化を演出</t>
+          <t>1.5秒後に5体・攻撃型で変化を加える</t>
         </is>
       </c>
       <c r="I41" s="2" t="n"/>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="H42" s="27" t="inlineStr">
         <is>
-          <t>3.0秒後・最終波で締め</t>
+          <t>3秒後に5体・継続プレッシャー（合計15体）</t>
         </is>
       </c>
       <c r="I42" s="2" t="n"/>
@@ -1896,7 +1896,7 @@
           <t>バトルヒント</t>
         </is>
       </c>
-      <c r="C58" s="27" t="inlineStr"/>
+      <c r="C58" s="18" t="inlineStr"/>
       <c r="D58" s="28" t="n"/>
       <c r="E58" s="28" t="n"/>
       <c r="F58" s="28" t="n"/>
@@ -1915,7 +1915,7 @@
           <t>ステージ説明文</t>
         </is>
       </c>
-      <c r="C59" s="27" t="inlineStr"/>
+      <c r="C59" s="18" t="inlineStr"/>
       <c r="D59" s="28" t="n"/>
       <c r="E59" s="28" t="n"/>
       <c r="F59" s="28" t="n"/>

</xml_diff>